<commit_message>
Two-layer spine + integrity gate + date-of-entry
Review grounded in actual schema (5 tables, not 4):
- property_units = physical master; tenancy_schedule_units = lease
  spine. Reassign physical facts (address, area, EPC, condition,
  use class) to property_units; they survive lease changes. Lease/
  income stays on tenancy. Fixes wrong-owner bug in prior matrix.
- Add integrity-gate-report.sql: read-only go/no-go reconciliation
  (null/dangling spine links, back-pointer + deal-id drift, multiple
  live deals per unit, duplicated-field drift, target-brand dupes).
  Finding: tenancy has no FK to property_units yet — must be added
  and back-filled.
- Surface date-of-entry (crm_deals.created_at, already exists).
- Add solicitor sub-journey rows (firm/contact/draft-lease/comments/
  engrossment/notes) — in schema, invisible in UI today.

101 facts, 48 detail-only.
</commit_message>
<xml_diff>
--- a/docs/unit-column-ownership.xlsx
+++ b/docs/unit-column-ownership.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="934" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1002" uniqueCount="219">
   <si>
     <t>Section</t>
   </si>
@@ -53,36 +53,51 @@
     <t>unit 1:1</t>
   </si>
   <si>
+    <t>property_units</t>
+  </si>
+  <si>
+    <t>read</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Physical. Today on tenancy.nia_sqft — migrate to property_units.</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>GIA sqft</t>
+  </si>
+  <si>
+    <t>Physical. Today on tenancy.gia_sqft — migrate.</t>
+  </si>
+  <si>
+    <t>ITZA sqft</t>
+  </si>
+  <si>
+    <t>Physical. Today on tenancy.itza_sqft — migrate.</t>
+  </si>
+  <si>
+    <t>Floor breakdown (bsmt/ground/first/other)</t>
+  </si>
+  <si>
+    <t>Physical. Detailed area split today on tenancy.</t>
+  </si>
+  <si>
+    <t>RENT</t>
+  </si>
+  <si>
+    <t>Passing rent pa (current tenant)</t>
+  </si>
+  <si>
     <t>tenancy</t>
   </si>
   <si>
     <t>edit</t>
   </si>
   <si>
-    <t>read</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>GIA sqft</t>
-  </si>
-  <si>
-    <t>ITZA sqft</t>
-  </si>
-  <si>
-    <t>Floor breakdown (bsmt/ground/first/other)</t>
-  </si>
-  <si>
-    <t>RENT</t>
-  </si>
-  <si>
-    <t>Passing rent pa (current tenant)</t>
-  </si>
-  <si>
     <t>Only changes on deal Complete. Sum = rent roll.</t>
   </si>
   <si>
@@ -206,12 +221,21 @@
     <t>EPC rating</t>
   </si>
   <si>
+    <t>Physical. Duplicated on property_units + available_units + tenancy today.</t>
+  </si>
+  <si>
     <t>Use class / permitted use</t>
   </si>
   <si>
+    <t>Physical/planning attribute. On property_units + available_units + tenancy today.</t>
+  </si>
+  <si>
     <t>Condition (Shell/CatA/CatB/Fitted...)</t>
   </si>
   <si>
+    <t>Physical. On property_units + available_units today.</t>
+  </si>
+  <si>
     <t>Location / UK region</t>
   </si>
   <si>
@@ -224,15 +248,27 @@
     <t>Address line</t>
   </si>
   <si>
+    <t>Already on property_units.unit_address.</t>
+  </si>
+  <si>
     <t>Postcode</t>
   </si>
   <si>
+    <t>Already on property_units.unit_postcode.</t>
+  </si>
+  <si>
     <t>UPRN</t>
   </si>
   <si>
+    <t>Already on property_units.unit_uprn.</t>
+  </si>
+  <si>
     <t>Free-text address fallback (non-PAF)</t>
   </si>
   <si>
+    <t>Already on property_units.unit_address_free_text.</t>
+  </si>
+  <si>
     <t>TENANT</t>
   </si>
   <si>
@@ -296,12 +332,24 @@
     <t>Target date</t>
   </si>
   <si>
-    <t>Instructed / exchanged / completed / invoiced dates</t>
+    <t>Date of entry (deal createdAt)</t>
+  </si>
+  <si>
+    <t>crm_deals (auto)</t>
+  </si>
+  <si>
+    <t>Already on crm_deals.created_at — surface + make sortable. 'How long open?'</t>
+  </si>
+  <si>
+    <t>Instructed (BGP put on deal) / target / exchanged / completed / invoiced dates</t>
   </si>
   <si>
     <t>read (to Completed)</t>
   </si>
   <si>
+    <t>instructed_at ≠ created_at ≠ solicitor_instructed_at — keep distinct.</t>
+  </si>
+  <si>
     <t>Pricing / yield (investment)</t>
   </si>
   <si>
@@ -377,6 +425,33 @@
     <t>MLRO risk-assessment PDF</t>
   </si>
   <si>
+    <t>SOLICITOR</t>
+  </si>
+  <si>
+    <t>Solicitor firm + contact</t>
+  </si>
+  <si>
+    <t>solicitor_firm / solicitor_contact.</t>
+  </si>
+  <si>
+    <t>Solicitor instructed date</t>
+  </si>
+  <si>
+    <t>solicitor_instructed_at.</t>
+  </si>
+  <si>
+    <t>Draft lease received / comments returned / engrossment dates</t>
+  </si>
+  <si>
+    <t>draft_lease_received_at / comments_returned_at / engrossment_at — drive Solicitors-stage progress.</t>
+  </si>
+  <si>
+    <t>Solicitor notes</t>
+  </si>
+  <si>
+    <t>solicitor_notes.</t>
+  </si>
+  <si>
     <t>INVOICING (Xero)</t>
   </si>
   <si>
@@ -575,7 +650,13 @@
     <t>RULES</t>
   </si>
   <si>
-    <t>Each fact has exactly one owner. Other surfaces read it via the spine link (tenancy_unit_id / deal_id).</t>
+    <t>TWO-LAYER SPINE: property_units owns PHYSICAL facts (address, area, EPC, condition, use class) — permanent, survives lease changes. tenancy_schedule_units owns LEASE/INCOME facts. Everyone reads through.</t>
+  </si>
+  <si>
+    <t>Each fact has exactly one owner. Other surfaces read it via the spine link (unit_id → property_units, tenancy_unit_id → tenancy, deal_id → crm_deals).</t>
+  </si>
+  <si>
+    <t>GAP: tenancy_schedule_units has no FK to property_units yet — must be added + back-filled (see integrity-gate-report.sql query 4).</t>
   </si>
   <si>
     <t>FOUR rents, all distinct: passing · ERV · quoting · agreed. Never collapsed.</t>
@@ -585,6 +666,9 @@
   </si>
   <si>
     <t>Letting Tracker is mostly a read-through view; editing happens at the source of truth.</t>
+  </si>
+  <si>
+    <t>Deal is born at Solicitors (WIP form), NOT on Add-Unit. Add-Unit writes property_units + tenancy_schedule_units.</t>
   </si>
 </sst>
 </file>
@@ -608,10 +692,6 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF15803D"/>
-    </font>
-    <font>
-      <b/>
       <color rgb="FF6B7280"/>
     </font>
     <font>
@@ -622,6 +702,10 @@
       <color rgb="FF6B7280"/>
     </font>
     <font/>
+    <font>
+      <b/>
+      <color rgb="FF15803D"/>
+    </font>
     <font>
       <b/>
       <color rgb="FFDC2626"/>
@@ -643,7 +727,7 @@
       <color rgb="FF7C3AED"/>
     </font>
   </fonts>
-  <fills count="19">
+  <fills count="20">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -702,6 +786,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFEDE9FE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFD1FAE5"/>
       </patternFill>
     </fill>
@@ -748,7 +837,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -768,16 +857,16 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -786,13 +875,13 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -801,19 +890,19 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -825,55 +914,61 @@
     <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1216,7 +1311,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J97"/>
+  <dimension ref="A1:J102"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1277,22 +1372,24 @@
       <c r="E2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="I2" s="6" t="s">
+      <c r="F2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J2" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="7"/>
     </row>
     <row r="3" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="7" t="s">
         <v>17</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -1307,26 +1404,28 @@
       <c r="E3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="5" t="s">
-        <v>15</v>
+      <c r="F3" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="I3" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J3" s="7"/>
+      <c r="H3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="4" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="7" t="s">
         <v>17</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>12</v>
@@ -1337,26 +1436,28 @@
       <c r="E4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="I4" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J4" s="7"/>
+      <c r="F4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="5" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="7" t="s">
         <v>17</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>12</v>
@@ -1367,50 +1468,52 @@
       <c r="E5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="5" t="s">
-        <v>15</v>
+      <c r="F5" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J5" s="7"/>
+      <c r="H5" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="6" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
-        <v>21</v>
+      <c r="A6" s="8" t="s">
+        <v>24</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>14</v>
+        <v>26</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="5" t="s">
-        <v>15</v>
+      <c r="G6" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J6" s="7" t="s">
-        <v>23</v>
+      <c r="I6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1418,31 +1521,31 @@
         <v>17</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>15</v>
+        <v>26</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I7" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J7" s="7" t="s">
-        <v>25</v>
+      <c r="I7" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1450,31 +1553,31 @@
         <v>17</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J8" s="7" t="s">
-        <v>28</v>
+        <v>32</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1482,31 +1585,31 @@
         <v>17</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J9" s="7" t="s">
-        <v>32</v>
+      <c r="F9" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1514,13 +1617,13 @@
         <v>17</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>34</v>
+        <v>38</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>39</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>17</v>
@@ -1531,14 +1634,14 @@
       <c r="G10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H10" s="5" t="s">
-        <v>15</v>
+      <c r="H10" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J10" s="7" t="s">
-        <v>36</v>
+        <v>40</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1546,43 +1649,43 @@
         <v>17</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>39</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="I11" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J11" s="7"/>
+        <v>39</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J11" s="6"/>
     </row>
     <row r="12" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
         <v>17</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C12" s="7" t="s">
-        <v>34</v>
-      </c>
       <c r="D12" s="2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>17</v>
@@ -1593,26 +1696,26 @@
       <c r="G12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H12" s="5" t="s">
-        <v>15</v>
+      <c r="H12" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J12" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J12" s="6"/>
     </row>
     <row r="13" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
         <v>17</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>34</v>
+        <v>45</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>39</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>17</v>
@@ -1623,56 +1726,56 @@
       <c r="G13" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H13" s="5" t="s">
-        <v>15</v>
+      <c r="H13" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J13" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J13" s="6"/>
     </row>
     <row r="14" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
         <v>17</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>14</v>
+        <v>26</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G14" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="I14" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J14" s="7"/>
+      <c r="G14" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J14" s="6"/>
     </row>
     <row r="15" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
         <v>17</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>17</v>
@@ -1683,26 +1786,26 @@
       <c r="G15" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H15" s="4" t="s">
-        <v>14</v>
+      <c r="H15" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J15" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J15" s="6"/>
     </row>
     <row r="16" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
         <v>17</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>17</v>
@@ -1713,59 +1816,59 @@
       <c r="G16" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H16" s="4" t="s">
-        <v>14</v>
+      <c r="H16" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J16" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J16" s="6"/>
     </row>
     <row r="17" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
         <v>17</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>14</v>
+        <v>26</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G17" s="5" t="s">
-        <v>15</v>
+      <c r="G17" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="H17" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I17" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J17" s="7"/>
+      <c r="I17" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J17" s="6"/>
     </row>
     <row r="18" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>14</v>
+        <v>26</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>17</v>
@@ -1776,146 +1879,146 @@
       <c r="H18" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I18" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J18" s="7"/>
+      <c r="I18" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J18" s="6"/>
     </row>
     <row r="19" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
         <v>17</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>14</v>
+        <v>26</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G19" s="5" t="s">
-        <v>15</v>
+      <c r="G19" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I19" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J19" s="7"/>
+      <c r="I19" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J19" s="6"/>
     </row>
     <row r="20" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
         <v>17</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>14</v>
+        <v>26</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G20" s="5" t="s">
-        <v>15</v>
+      <c r="G20" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I20" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J20" s="7"/>
+      <c r="I20" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J20" s="6"/>
     </row>
     <row r="21" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
         <v>17</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>14</v>
+        <v>26</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G21" s="5" t="s">
-        <v>15</v>
+      <c r="G21" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I21" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J21" s="7"/>
+      <c r="I21" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J21" s="6"/>
     </row>
     <row r="22" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
         <v>17</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>14</v>
+        <v>26</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G22" s="5" t="s">
-        <v>15</v>
+      <c r="G22" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="H22" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I22" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J22" s="7"/>
+      <c r="I22" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J22" s="6"/>
     </row>
     <row r="23" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
         <v>17</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>14</v>
+        <v>26</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>17</v>
@@ -1926,116 +2029,116 @@
       <c r="H23" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I23" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J23" s="7"/>
+      <c r="I23" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J23" s="6"/>
     </row>
     <row r="24" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
         <v>17</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>34</v>
+        <v>57</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>39</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>43</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G24" s="5" t="s">
-        <v>38</v>
+      <c r="G24" s="4" t="s">
+        <v>43</v>
       </c>
       <c r="H24" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I24" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J24" s="7"/>
+      <c r="I24" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J24" s="6"/>
     </row>
     <row r="25" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
         <v>17</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F25" s="5" t="s">
-        <v>15</v>
+      <c r="F25" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H25" s="4" t="s">
-        <v>14</v>
+      <c r="H25" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I25" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J25" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J25" s="6"/>
     </row>
     <row r="26" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="13" t="s">
         <v>17</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F26" s="5" t="s">
-        <v>15</v>
+      <c r="F26" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H26" s="4" t="s">
-        <v>14</v>
+      <c r="H26" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J26" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J26" s="6"/>
     </row>
     <row r="27" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>14</v>
+        <v>32</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>17</v>
@@ -2046,137 +2149,137 @@
       <c r="H27" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I27" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J27" s="7"/>
+      <c r="I27" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J27" s="6"/>
     </row>
     <row r="28" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="15" t="s">
         <v>17</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>14</v>
+        <v>32</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="F28" s="16" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="G28" s="16" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="H28" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I28" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J28" s="7"/>
+      <c r="I28" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J28" s="6"/>
     </row>
     <row r="29" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="15" t="s">
         <v>17</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F29" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G29" s="5" t="s">
-        <v>15</v>
+        <v>32</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="H29" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I29" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J29" s="7"/>
+      <c r="I29" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J29" s="6"/>
     </row>
     <row r="30" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="15" t="s">
         <v>17</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F30" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G30" s="5" t="s">
-        <v>15</v>
+      <c r="F30" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="H30" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I30" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J30" s="7"/>
+      <c r="I30" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J30" s="6"/>
     </row>
     <row r="31" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="15" t="s">
         <v>17</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F31" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G31" s="5" t="s">
-        <v>15</v>
+      <c r="F31" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="H31" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I31" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J31" s="7"/>
+      <c r="I31" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J31" s="6"/>
     </row>
     <row r="32" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="15" t="s">
         <v>17</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>12</v>
@@ -2187,26 +2290,28 @@
       <c r="E32" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F32" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G32" s="5" t="s">
-        <v>15</v>
+      <c r="F32" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="H32" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I32" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J32" s="7"/>
+      <c r="I32" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J32" s="6" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="33" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="15" t="s">
         <v>17</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>12</v>
@@ -2217,38 +2322,40 @@
       <c r="E33" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F33" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G33" s="5" t="s">
-        <v>15</v>
+      <c r="F33" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="H33" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I33" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J33" s="7"/>
+      <c r="I33" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J33" s="6" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="34" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="15" t="s">
         <v>17</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>61</v>
+        <v>13</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F34" s="2" t="s">
-        <v>17</v>
+      <c r="F34" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="G34" s="2" t="s">
         <v>17</v>
@@ -2256,29 +2363,31 @@
       <c r="H34" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I34" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J34" s="7"/>
+      <c r="I34" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J34" s="6" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="35" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="15" t="s">
         <v>17</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F35" s="4" t="s">
-        <v>14</v>
+      <c r="F35" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>17</v>
@@ -2287,22 +2396,22 @@
         <v>17</v>
       </c>
       <c r="I35" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J35" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J35" s="6"/>
     </row>
     <row r="36" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="15" t="s">
         <v>17</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>17</v>
@@ -2317,16 +2426,16 @@
         <v>17</v>
       </c>
       <c r="I36" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J36" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J36" s="6"/>
     </row>
     <row r="37" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="17" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>12</v>
@@ -2337,26 +2446,28 @@
       <c r="E37" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F37" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G37" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H37" s="5" t="s">
-        <v>15</v>
+      <c r="F37" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G37" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H37" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="I37" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J37" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J37" s="6" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="38" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="18" t="s">
         <v>17</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>12</v>
@@ -2367,26 +2478,28 @@
       <c r="E38" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F38" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G38" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H38" s="5" t="s">
-        <v>15</v>
+      <c r="F38" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H38" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="I38" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J38" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J38" s="6" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="39" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="18" t="s">
         <v>17</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>12</v>
@@ -2403,20 +2516,22 @@
       <c r="G39" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H39" s="5" t="s">
-        <v>15</v>
+      <c r="H39" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="I39" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J39" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J39" s="6" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="40" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="18" t="s">
         <v>17</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>12</v>
@@ -2433,146 +2548,148 @@
       <c r="G40" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H40" s="5" t="s">
-        <v>15</v>
+      <c r="H40" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J40" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J40" s="6" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="41" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="19" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>14</v>
+        <v>26</v>
+      </c>
+      <c r="E41" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="F41" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G41" s="5" t="s">
-        <v>15</v>
+      <c r="G41" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="H41" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I41" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J41" s="7"/>
+      <c r="I41" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J41" s="6"/>
     </row>
     <row r="42" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E42" s="4" t="s">
-        <v>14</v>
+        <v>26</v>
+      </c>
+      <c r="E42" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="F42" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G42" s="5" t="s">
-        <v>15</v>
+      <c r="G42" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="H42" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I42" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J42" s="7"/>
+      <c r="I42" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J42" s="6"/>
     </row>
     <row r="43" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E43" s="4" t="s">
-        <v>14</v>
+        <v>26</v>
+      </c>
+      <c r="E43" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="F43" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G43" s="5" t="s">
-        <v>15</v>
+      <c r="G43" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="H43" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I43" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J43" s="7"/>
+      <c r="I43" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J43" s="6"/>
     </row>
     <row r="44" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E44" s="4" t="s">
-        <v>14</v>
+        <v>26</v>
+      </c>
+      <c r="E44" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="F44" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G44" s="5" t="s">
-        <v>15</v>
+      <c r="G44" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="H44" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I44" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J44" s="7"/>
+      <c r="I44" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J44" s="6"/>
     </row>
     <row r="45" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="21" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>17</v>
@@ -2583,56 +2700,56 @@
       <c r="G45" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H45" s="4" t="s">
-        <v>14</v>
+      <c r="H45" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I45" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J45" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J45" s="6"/>
     </row>
     <row r="46" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="22" t="s">
         <v>17</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F46" s="4" t="s">
-        <v>14</v>
+      <c r="F46" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="G46" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H46" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="I46" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J46" s="7"/>
+      <c r="H46" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I46" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J46" s="6"/>
     </row>
     <row r="47" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="22" t="s">
         <v>17</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>17</v>
@@ -2643,116 +2760,116 @@
       <c r="G47" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H47" s="4" t="s">
-        <v>14</v>
+      <c r="H47" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I47" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J47" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J47" s="6"/>
     </row>
     <row r="48" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="22" t="s">
         <v>17</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E48" s="23" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="F48" s="23" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="G48" s="23" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="H48" s="23" t="s">
-        <v>83</v>
-      </c>
-      <c r="I48" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J48" s="7"/>
+        <v>95</v>
+      </c>
+      <c r="I48" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J48" s="6"/>
     </row>
     <row r="49" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="22" t="s">
         <v>17</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F49" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G49" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H49" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="I49" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J49" s="7"/>
+      <c r="F49" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="G49" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H49" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I49" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J49" s="6"/>
     </row>
     <row r="50" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="22" t="s">
         <v>17</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F50" s="5" t="s">
-        <v>15</v>
+      <c r="F50" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="G50" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H50" s="4" t="s">
-        <v>14</v>
+      <c r="H50" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I50" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J50" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J50" s="6"/>
     </row>
     <row r="51" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="22" t="s">
         <v>17</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>17</v>
@@ -2763,26 +2880,26 @@
       <c r="G51" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H51" s="4" t="s">
-        <v>14</v>
+      <c r="H51" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I51" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J51" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J51" s="6"/>
     </row>
     <row r="52" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="22" t="s">
         <v>17</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>17</v>
@@ -2793,176 +2910,180 @@
       <c r="G52" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H52" s="4" t="s">
-        <v>14</v>
+      <c r="H52" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J52" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J52" s="6"/>
     </row>
     <row r="53" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="22" t="s">
         <v>17</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F53" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G53" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H53" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="I53" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J53" s="7"/>
+      <c r="F53" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G53" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H53" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I53" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J53" s="6"/>
     </row>
     <row r="54" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="22" t="s">
         <v>17</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="C54" s="24" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F54" s="16" t="s">
-        <v>92</v>
-      </c>
-      <c r="G54" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H54" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="I54" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J54" s="7"/>
+        <v>104</v>
+      </c>
+      <c r="G54" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H54" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I54" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J54" s="6"/>
     </row>
     <row r="55" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="22" t="s">
         <v>17</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F55" s="4" t="s">
-        <v>14</v>
+      <c r="F55" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="G55" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H55" s="4" t="s">
-        <v>14</v>
+      <c r="H55" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J55" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J55" s="6"/>
     </row>
     <row r="56" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="22" t="s">
         <v>17</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>31</v>
+        <v>107</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F56" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G56" s="5" t="s">
-        <v>95</v>
+      <c r="F56" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>17</v>
       </c>
       <c r="H56" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="I56" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J56" s="7"/>
+      <c r="I56" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J56" s="6" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="57" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="22" t="s">
         <v>17</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F57" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G57" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H57" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="I57" s="11" t="s">
+      <c r="F57" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G57" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="H57" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I57" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J57" s="6" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C58" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="J57" s="7"/>
-    </row>
-    <row r="58" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="25" t="s">
-        <v>97</v>
-      </c>
-      <c r="B58" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>30</v>
-      </c>
       <c r="D58" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>17</v>
@@ -2973,26 +3094,26 @@
       <c r="G58" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H58" s="4" t="s">
-        <v>14</v>
+      <c r="H58" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I58" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="J58" s="6"/>
+    </row>
+    <row r="59" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C59" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="J58" s="7"/>
-    </row>
-    <row r="59" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="26" t="s">
-        <v>17</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>30</v>
-      </c>
       <c r="D59" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>17</v>
@@ -3003,26 +3124,26 @@
       <c r="G59" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H59" s="4" t="s">
-        <v>14</v>
+      <c r="H59" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J59" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J59" s="6"/>
     </row>
     <row r="60" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="26" t="s">
         <v>17</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>17</v>
@@ -3033,26 +3154,26 @@
       <c r="G60" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H60" s="4" t="s">
-        <v>14</v>
+      <c r="H60" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I60" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J60" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J60" s="6"/>
     </row>
     <row r="61" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="26" t="s">
         <v>17</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E61" s="2" t="s">
         <v>17</v>
@@ -3063,26 +3184,26 @@
       <c r="G61" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H61" s="4" t="s">
-        <v>14</v>
+      <c r="H61" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J61" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J61" s="6"/>
     </row>
     <row r="62" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="26" t="s">
         <v>17</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>17</v>
@@ -3093,146 +3214,146 @@
       <c r="G62" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H62" s="4" t="s">
-        <v>14</v>
+      <c r="H62" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I62" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="J62" s="6"/>
+    </row>
+    <row r="63" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C63" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="J62" s="7"/>
-    </row>
-    <row r="63" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="27" t="s">
-        <v>103</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="C63" s="2" t="s">
-        <v>30</v>
-      </c>
       <c r="D63" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E63" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F63" s="4" t="s">
-        <v>14</v>
+      <c r="F63" s="2" t="s">
+        <v>17</v>
       </c>
       <c r="G63" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H63" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="I63" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J63" s="7"/>
+      <c r="H63" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I63" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="J63" s="6"/>
     </row>
     <row r="64" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="28" t="s">
-        <v>17</v>
+      <c r="A64" s="27" t="s">
+        <v>119</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E64" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F64" s="4" t="s">
-        <v>14</v>
+      <c r="F64" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="G64" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H64" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="I64" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J64" s="7"/>
+      <c r="H64" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I64" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J64" s="6"/>
     </row>
     <row r="65" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="28" t="s">
         <v>17</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E65" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F65" s="4" t="s">
-        <v>14</v>
+      <c r="F65" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="G65" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H65" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="I65" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J65" s="7"/>
+      <c r="H65" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I65" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="J65" s="6"/>
     </row>
     <row r="66" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="28" t="s">
         <v>17</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E66" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F66" s="5" t="s">
-        <v>15</v>
+      <c r="F66" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="G66" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H66" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="I66" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J66" s="7"/>
+      <c r="H66" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I66" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J66" s="6"/>
     </row>
     <row r="67" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="28" t="s">
         <v>17</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="C67" s="24" t="s">
-        <v>91</v>
+        <v>123</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E67" s="2" t="s">
         <v>17</v>
@@ -3247,118 +3368,116 @@
         <v>14</v>
       </c>
       <c r="I67" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="J67" s="6"/>
+    </row>
+    <row r="68" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C68" s="24" t="s">
+        <v>103</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F68" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H68" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I68" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="J68" s="6" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="19" t="s">
+        <v>126</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C69" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="J67" s="7" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="68" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="19" t="s">
-        <v>110</v>
-      </c>
-      <c r="B68" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C68" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D68" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E68" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F68" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G68" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H68" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="I68" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J68" s="7" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="69" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="20" t="s">
-        <v>17</v>
-      </c>
-      <c r="B69" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="C69" s="2" t="s">
-        <v>30</v>
-      </c>
       <c r="D69" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E69" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F69" s="4" t="s">
-        <v>14</v>
+      <c r="F69" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="G69" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H69" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="I69" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J69" s="7"/>
+      <c r="H69" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I69" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J69" s="6" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="70" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="C70" s="24" t="s">
-        <v>91</v>
+        <v>129</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>115</v>
+        <v>36</v>
       </c>
       <c r="E70" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F70" s="2" t="s">
-        <v>17</v>
+      <c r="F70" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="G70" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H70" s="4" t="s">
-        <v>14</v>
+      <c r="H70" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I70" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J70" s="7" t="s">
-        <v>116</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="J70" s="6"/>
     </row>
     <row r="71" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="C71" s="24" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>115</v>
+        <v>131</v>
       </c>
       <c r="E71" s="2" t="s">
         <v>17</v>
@@ -3369,26 +3488,28 @@
       <c r="G71" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H71" s="4" t="s">
-        <v>14</v>
+      <c r="H71" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I71" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J71" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J71" s="6" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="72" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
       <c r="C72" s="24" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>115</v>
+        <v>131</v>
       </c>
       <c r="E72" s="2" t="s">
         <v>17</v>
@@ -3399,26 +3520,26 @@
       <c r="G72" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H72" s="5" t="s">
-        <v>15</v>
+      <c r="H72" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I72" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J72" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J72" s="6"/>
     </row>
     <row r="73" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="C73" s="2" t="s">
-        <v>30</v>
+        <v>134</v>
+      </c>
+      <c r="C73" s="24" t="s">
+        <v>103</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>115</v>
+        <v>131</v>
       </c>
       <c r="E73" s="2" t="s">
         <v>17</v>
@@ -3429,26 +3550,26 @@
       <c r="G73" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H73" s="5" t="s">
-        <v>15</v>
+      <c r="H73" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="I73" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J73" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J73" s="6"/>
     </row>
     <row r="74" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>115</v>
+        <v>131</v>
       </c>
       <c r="E74" s="2" t="s">
         <v>17</v>
@@ -3459,26 +3580,26 @@
       <c r="G74" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H74" s="5" t="s">
-        <v>15</v>
+      <c r="H74" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="I74" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="J74" s="6"/>
+    </row>
+    <row r="75" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C75" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="J74" s="7"/>
-    </row>
-    <row r="75" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="29" t="s">
-        <v>121</v>
-      </c>
-      <c r="B75" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="C75" s="24" t="s">
-        <v>91</v>
-      </c>
       <c r="D75" s="2" t="s">
-        <v>31</v>
+        <v>131</v>
       </c>
       <c r="E75" s="2" t="s">
         <v>17</v>
@@ -3493,24 +3614,22 @@
         <v>14</v>
       </c>
       <c r="I75" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="J75" s="6"/>
+    </row>
+    <row r="76" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A76" s="29" t="s">
+        <v>137</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C76" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="J75" s="7" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="76" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="30" t="s">
-        <v>17</v>
-      </c>
-      <c r="B76" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="C76" s="2" t="s">
-        <v>30</v>
-      </c>
       <c r="D76" s="2" t="s">
-        <v>125</v>
+        <v>36</v>
       </c>
       <c r="E76" s="2" t="s">
         <v>17</v>
@@ -3521,26 +3640,28 @@
       <c r="G76" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H76" s="5" t="s">
-        <v>15</v>
+      <c r="H76" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I76" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J76" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J76" s="6" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="77" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="30" t="s">
         <v>17</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E77" s="2" t="s">
         <v>17</v>
@@ -3551,26 +3672,28 @@
       <c r="G77" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H77" s="4" t="s">
-        <v>14</v>
+      <c r="H77" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I77" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J77" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J77" s="6" t="s">
+        <v>141</v>
+      </c>
     </row>
     <row r="78" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="30" t="s">
         <v>17</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>127</v>
+        <v>142</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>125</v>
+        <v>36</v>
       </c>
       <c r="E78" s="2" t="s">
         <v>17</v>
@@ -3581,26 +3704,28 @@
       <c r="G78" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H78" s="4" t="s">
-        <v>14</v>
+      <c r="H78" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I78" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="J78" s="6" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="30" t="s">
+        <v>17</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C79" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="J78" s="7"/>
-    </row>
-    <row r="79" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="31" t="s">
-        <v>128</v>
-      </c>
-      <c r="B79" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="C79" s="32" t="s">
-        <v>130</v>
-      </c>
       <c r="D79" s="2" t="s">
-        <v>131</v>
+        <v>36</v>
       </c>
       <c r="E79" s="2" t="s">
         <v>17</v>
@@ -3611,120 +3736,120 @@
       <c r="G79" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H79" s="5" t="s">
-        <v>15</v>
+      <c r="H79" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I79" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="J79" s="6" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="31" t="s">
+        <v>146</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C80" s="24" t="s">
+        <v>103</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E80" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F80" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G80" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H80" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I80" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="J80" s="6" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C81" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="J79" s="7"/>
-    </row>
-    <row r="80" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="33" t="s">
-        <v>17</v>
-      </c>
-      <c r="B80" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="C80" s="32" t="s">
-        <v>130</v>
-      </c>
-      <c r="D80" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="E80" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F80" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G80" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H80" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="I80" s="11" t="s">
+      <c r="D81" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="E81" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F81" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G81" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H81" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I81" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="J81" s="6"/>
+    </row>
+    <row r="82" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A82" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C82" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="J80" s="7"/>
-    </row>
-    <row r="81" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="34" t="s">
-        <v>133</v>
-      </c>
-      <c r="B81" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="C81" s="24" t="s">
-        <v>91</v>
-      </c>
-      <c r="D81" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="E81" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F81" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G81" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H81" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="I81" s="11" t="s">
+      <c r="D82" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E82" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F82" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G82" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H82" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I82" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="J82" s="6"/>
+    </row>
+    <row r="83" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A83" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C83" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="J81" s="7" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="82" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="35" t="s">
-        <v>17</v>
-      </c>
-      <c r="B82" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="C82" s="24" t="s">
-        <v>91</v>
-      </c>
-      <c r="D82" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="E82" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F82" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G82" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H82" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="I82" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J82" s="7" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="83" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="35" t="s">
-        <v>17</v>
-      </c>
-      <c r="B83" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="C83" s="32" t="s">
-        <v>139</v>
-      </c>
       <c r="D83" s="2" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="E83" s="2" t="s">
         <v>17</v>
@@ -3735,26 +3860,26 @@
       <c r="G83" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H83" s="5" t="s">
-        <v>15</v>
+      <c r="H83" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="I83" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J83" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J83" s="6"/>
     </row>
     <row r="84" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="36" t="s">
-        <v>141</v>
+      <c r="A84" s="33" t="s">
+        <v>153</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="C84" s="32" t="s">
-        <v>139</v>
+        <v>154</v>
+      </c>
+      <c r="C84" s="34" t="s">
+        <v>155</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
       <c r="E84" s="2" t="s">
         <v>17</v>
@@ -3769,116 +3894,116 @@
         <v>14</v>
       </c>
       <c r="I84" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="J84" s="7"/>
+        <v>40</v>
+      </c>
+      <c r="J84" s="6"/>
     </row>
     <row r="85" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="37" t="s">
+      <c r="A85" s="35" t="s">
         <v>17</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="C85" s="24" t="s">
-        <v>145</v>
+        <v>157</v>
+      </c>
+      <c r="C85" s="34" t="s">
+        <v>155</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="E85" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F85" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G85" s="5" t="s">
-        <v>15</v>
+      <c r="F85" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G85" s="2" t="s">
+        <v>17</v>
       </c>
       <c r="H85" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="I85" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J85" s="7"/>
+      <c r="I85" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="J85" s="6"/>
     </row>
     <row r="86" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="38" t="s">
-        <v>147</v>
+      <c r="A86" s="36" t="s">
+        <v>158</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>148</v>
+        <v>159</v>
       </c>
       <c r="C86" s="24" t="s">
-        <v>145</v>
+        <v>103</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>149</v>
+        <v>160</v>
       </c>
       <c r="E86" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F86" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G86" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H86" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I86" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J86" s="7" t="s">
-        <v>150</v>
+      <c r="F86" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G86" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H86" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I86" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="J86" s="6" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="87" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="38" t="s">
-        <v>151</v>
+      <c r="A87" s="37" t="s">
+        <v>17</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
       <c r="C87" s="24" t="s">
-        <v>145</v>
+        <v>103</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="E87" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F87" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G87" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H87" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I87" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J87" s="7" t="s">
-        <v>154</v>
+      <c r="F87" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G87" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H87" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I87" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="J87" s="6" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="88" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="39" t="s">
-        <v>155</v>
+      <c r="A88" s="37" t="s">
+        <v>17</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="C88" s="2" t="s">
-        <v>12</v>
+        <v>163</v>
+      </c>
+      <c r="C88" s="34" t="s">
+        <v>164</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="E88" s="2" t="s">
         <v>17</v>
@@ -3886,29 +4011,29 @@
       <c r="F88" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G88" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H88" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I88" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J88" s="7"/>
+      <c r="G88" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H88" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I88" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="J88" s="6"/>
     </row>
     <row r="89" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="40" t="s">
-        <v>17</v>
+      <c r="A89" s="38" t="s">
+        <v>166</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="C89" s="2" t="s">
-        <v>12</v>
+        <v>167</v>
+      </c>
+      <c r="C89" s="34" t="s">
+        <v>164</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>157</v>
+        <v>168</v>
       </c>
       <c r="E89" s="2" t="s">
         <v>17</v>
@@ -3916,67 +4041,65 @@
       <c r="F89" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G89" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H89" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I89" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J89" s="7"/>
+      <c r="G89" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H89" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I89" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="J89" s="6"/>
     </row>
     <row r="90" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="40" t="s">
+      <c r="A90" s="39" t="s">
         <v>17</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="C90" s="2" t="s">
-        <v>12</v>
+        <v>169</v>
+      </c>
+      <c r="C90" s="24" t="s">
+        <v>170</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>157</v>
+        <v>171</v>
       </c>
       <c r="E90" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F90" s="4" t="s">
-        <v>14</v>
+      <c r="F90" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="G90" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H90" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I90" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J90" s="7" t="s">
-        <v>160</v>
-      </c>
+      <c r="H90" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="I90" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J90" s="6"/>
     </row>
     <row r="91" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="40" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="C91" s="2" t="s">
-        <v>12</v>
+        <v>173</v>
+      </c>
+      <c r="C91" s="24" t="s">
+        <v>170</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>157</v>
+        <v>174</v>
       </c>
       <c r="E91" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F91" s="4" t="s">
-        <v>14</v>
+      <c r="F91" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="G91" s="4" t="s">
         <v>14</v>
@@ -3984,190 +4107,346 @@
       <c r="H91" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I91" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J91" s="7"/>
+      <c r="I91" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J91" s="6" t="s">
+        <v>175</v>
+      </c>
     </row>
     <row r="92" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A92" s="41" t="s">
-        <v>162</v>
+      <c r="A92" s="40" t="s">
+        <v>176</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="C92" s="2" t="s">
-        <v>12</v>
+        <v>177</v>
+      </c>
+      <c r="C92" s="24" t="s">
+        <v>170</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E92" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F92" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G92" s="2" t="s">
-        <v>17</v>
+        <v>178</v>
+      </c>
+      <c r="E92" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F92" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="G92" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="H92" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I92" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J92" s="7"/>
+      <c r="I92" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J92" s="6" t="s">
+        <v>179</v>
+      </c>
     </row>
     <row r="93" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="42" t="s">
-        <v>17</v>
+      <c r="A93" s="41" t="s">
+        <v>180</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>164</v>
+        <v>181</v>
       </c>
       <c r="C93" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E93" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F93" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G93" s="5" t="s">
-        <v>15</v>
+        <v>182</v>
+      </c>
+      <c r="E93" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F93" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G93" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="H93" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I93" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J93" s="7"/>
+      <c r="I93" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J93" s="6"/>
     </row>
     <row r="94" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="42" t="s">
         <v>17</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>165</v>
+        <v>183</v>
       </c>
       <c r="C94" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E94" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F94" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G94" s="5" t="s">
-        <v>15</v>
+        <v>182</v>
+      </c>
+      <c r="E94" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F94" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G94" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="H94" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I94" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J94" s="7"/>
+      <c r="I94" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J94" s="6"/>
     </row>
     <row r="95" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="42" t="s">
         <v>17</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>166</v>
+        <v>184</v>
       </c>
       <c r="C95" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E95" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F95" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G95" s="5" t="s">
-        <v>15</v>
+        <v>182</v>
+      </c>
+      <c r="E95" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F95" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="G95" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="H95" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I95" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J95" s="7"/>
+      <c r="I95" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J95" s="6" t="s">
+        <v>185</v>
+      </c>
     </row>
     <row r="96" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="42" t="s">
         <v>17</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>167</v>
+        <v>186</v>
       </c>
       <c r="C96" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E96" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F96" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G96" s="5" t="s">
-        <v>15</v>
+        <v>182</v>
+      </c>
+      <c r="E96" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F96" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="G96" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="H96" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I96" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J96" s="7"/>
+      <c r="I96" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J96" s="6"/>
     </row>
     <row r="97" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="42" t="s">
-        <v>17</v>
+      <c r="A97" s="43" t="s">
+        <v>187</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="C97" s="7" t="s">
-        <v>34</v>
+        <v>188</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E97" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F97" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="G97" s="5" t="s">
-        <v>38</v>
+        <v>26</v>
+      </c>
+      <c r="E97" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F97" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G97" s="2" t="s">
+        <v>17</v>
       </c>
       <c r="H97" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I97" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J97" s="7"/>
+      <c r="I97" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J97" s="6"/>
+    </row>
+    <row r="98" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A98" s="44" t="s">
+        <v>17</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E98" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F98" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G98" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H98" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I98" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J98" s="6"/>
+    </row>
+    <row r="99" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A99" s="44" t="s">
+        <v>17</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D99" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E99" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F99" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G99" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H99" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I99" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J99" s="6"/>
+    </row>
+    <row r="100" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A100" s="44" t="s">
+        <v>17</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D100" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E100" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F100" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G100" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H100" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I100" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J100" s="6"/>
+    </row>
+    <row r="101" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A101" s="44" t="s">
+        <v>17</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E101" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F101" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G101" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H101" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I101" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J101" s="6"/>
+    </row>
+    <row r="102" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A102" s="44" t="s">
+        <v>17</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C102" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E102" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F102" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="G102" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="H102" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I102" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J102" s="6"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
@@ -4178,59 +4457,59 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="95" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="43" t="s">
-        <v>169</v>
-      </c>
-      <c r="B1" s="43" t="s">
-        <v>170</v>
+    <row r="1" spans="1:2" s="45" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="45" t="s">
+        <v>194</v>
+      </c>
+      <c r="B1" s="45" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B2" t="s">
-        <v>171</v>
+        <v>196</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>172</v>
+        <v>197</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="B4" t="s">
-        <v>173</v>
+        <v>198</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="B5" t="s">
-        <v>174</v>
+        <v>199</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -4241,11 +4520,11 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:2" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="43" t="s">
-        <v>176</v>
-      </c>
-      <c r="B8" s="43" t="s">
+    <row r="8" spans="1:2" s="45" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="45" t="s">
+        <v>201</v>
+      </c>
+      <c r="B8" s="45" t="s">
         <v>17</v>
       </c>
     </row>
@@ -4254,39 +4533,39 @@
         <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>177</v>
+        <v>202</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B10" t="s">
-        <v>178</v>
+        <v>203</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="B11" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>181</v>
+        <v>206</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>139</v>
+        <v>164</v>
       </c>
       <c r="B13" t="s">
-        <v>182</v>
+        <v>207</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -4297,28 +4576,28 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:2" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="43" t="s">
+    <row r="15" spans="1:2" s="45" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="43" t="s">
+      <c r="B15" s="45" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>183</v>
+        <v>208</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>184</v>
+        <v>209</v>
       </c>
       <c r="B17" t="s">
-        <v>185</v>
+        <v>210</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -4329,11 +4608,11 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:2" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="43" t="s">
-        <v>186</v>
-      </c>
-      <c r="B19" s="43" t="s">
+    <row r="19" spans="1:2" s="45" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="45" t="s">
+        <v>211</v>
+      </c>
+      <c r="B19" s="45" t="s">
         <v>17</v>
       </c>
     </row>
@@ -4342,7 +4621,7 @@
         <v>17</v>
       </c>
       <c r="B20" t="s">
-        <v>187</v>
+        <v>212</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -4350,7 +4629,7 @@
         <v>17</v>
       </c>
       <c r="B21" t="s">
-        <v>188</v>
+        <v>213</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -4358,7 +4637,7 @@
         <v>17</v>
       </c>
       <c r="B22" t="s">
-        <v>189</v>
+        <v>214</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -4366,7 +4645,31 @@
         <v>17</v>
       </c>
       <c r="B23" t="s">
-        <v>190</v>
+        <v>215</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>17</v>
+      </c>
+      <c r="B24" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>17</v>
+      </c>
+      <c r="B25" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>17</v>
+      </c>
+      <c r="B26" t="s">
+        <v>218</v>
       </c>
     </row>
   </sheetData>

</xml_diff>